<commit_message>
adjust repoty terima secondary luar - adjust date from & to - add a few notes on excel
</commit_message>
<xml_diff>
--- a/public/assets/example/contoh-import-terima-secondary-luar.xlsx
+++ b/public/assets/example/contoh-import-terima-secondary-luar.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Tanggal</t>
   </si>
@@ -56,6 +56,28 @@
     <t>Qty</t>
   </si>
   <si>
+    <r>
+      <t xml:space="preserve">*Baris pertama ini </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t>jangan</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> dihapus/diubah</t>
+    </r>
+  </si>
+  <si>
     <t>CLB/0326/020</t>
   </si>
   <si>
@@ -77,16 +99,38 @@
     <t>DPN EMBRO</t>
   </si>
   <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>019 COOL GREY</t>
-  </si>
-  <si>
-    <t>S</t>
-  </si>
-  <si>
-    <t>XXL</t>
+    <t>*Baris ke-dua hanya data contoh, silahkan hapus lalu isi kembali dengan data yang asli</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">*Pastikan </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t>No. WS, Buyer, Style, Color, Size, Panel, Part</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> di-isi dengan </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t>sesuai</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -99,7 +143,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -261,6 +305,12 @@
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="34">
@@ -732,13 +782,17 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="58" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1272,8 +1326,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="5"/>
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="2"/>
   <cols>
     <col min="1" max="1" width="10.2857142857143" customWidth="1"/>
     <col min="2" max="2" width="14.8571428571429" customWidth="1"/>
@@ -1282,11 +1336,12 @@
     <col min="5" max="5" width="37.5714285714286" customWidth="1"/>
     <col min="6" max="6" width="5.14285714285714" customWidth="1"/>
     <col min="7" max="7" width="8" customWidth="1"/>
-    <col min="8" max="8" width="22.4285714285714" customWidth="1"/>
+    <col min="8" max="8" width="26.4285714285714" customWidth="1"/>
     <col min="9" max="9" width="5.57142857142857" customWidth="1"/>
+    <col min="10" max="10" width="94.4285714285714" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21" customHeight="1" spans="1:9">
+    <row r="1" ht="21" customHeight="1" spans="1:10">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1314,150 +1369,45 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:9">
-      <c r="A2" s="2">
+    <row r="2" spans="1:10">
+      <c r="A2" s="3">
         <v>46234</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="F2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="G2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="3">
+      <c r="H2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="4">
         <v>4</v>
       </c>
+      <c r="J2" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="3" spans="1:9">
-      <c r="A3" s="2">
-        <v>46234</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" s="3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="A4" s="2">
-        <v>46234</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I4" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5" s="2">
-        <v>46234</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F5" s="3" t="s">
+    <row r="3" ht="15.75" spans="1:10">
+      <c r="J3" s="5" t="s">
         <v>18</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I5" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="A6" s="2">
-        <v>46234</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I6" s="3">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>